<commit_message>
minimum_tax: Korea IIR/UTPR adoption in 2025
</commit_message>
<xml_diff>
--- a/final_outputs/rank_changes_2026.xlsx
+++ b/final_outputs/rank_changes_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\international-tax-competitiveness-index\final_outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF63DDFF-33A5-4048-B5A2-12BFA842C1B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD23A382-BF4F-4C6A-84B4-4A1AEF2DF6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{789578D4-DC63-490E-BC13-CED8D82346B8}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{67B8F1EA-256E-450E-AACF-1BF85E979D51}"/>
   </bookViews>
   <sheets>
     <sheet name="Rank changes 2026" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="102">
   <si>
     <t>Country</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Estonia</t>
   </si>
   <si>
-    <t>Corporate alt. minimum 1 -&gt; 0; top PIT rate 20% -&gt; 22%</t>
-  </si>
-  <si>
     <t>CFC active 0 -&gt; 0.5 (ATAD Model B)</t>
   </si>
   <si>
@@ -86,27 +83,18 @@
     <t>New Zealand</t>
   </si>
   <si>
-    <t>Corporate alt. minimum 0 -&gt; 1</t>
-  </si>
-  <si>
     <t>Dividend WHT 30% -&gt; 0 (imputation netted out)</t>
   </si>
   <si>
     <t>Switzerland</t>
   </si>
   <si>
-    <t>Digital services tax 1 -&gt; 0</t>
-  </si>
-  <si>
     <t>Revenue measures now shares of tax revenue, not GDP (was 2nd highest)</t>
   </si>
   <si>
     <t>Lithuania</t>
   </si>
   <si>
-    <t>Corporate rate 16% -&gt; 17%; dividend WHT 16% -&gt; 17%; machinery and intangibles cost recovery to 100%; R&amp;D credit up</t>
-  </si>
-  <si>
     <t>Luxembourg</t>
   </si>
   <si>
@@ -119,9 +107,6 @@
     <t>Czech Republic</t>
   </si>
   <si>
-    <t>Capital gains rate 23% -&gt; 0</t>
-  </si>
-  <si>
     <t>Israel</t>
   </si>
   <si>
@@ -143,13 +128,7 @@
     <t>Hungary</t>
   </si>
   <si>
-    <t>Turnover tax revenue 45% -&gt; 51%</t>
-  </si>
-  <si>
-    <t>Corporate alt. minimum 1 -&gt; 2; digital services tax 1 -&gt; 0; R&amp;D credit up</t>
-  </si>
-  <si>
-    <t>New turnover tax variable (highest value in the Index); CFC active 0 -&gt; 0.5</t>
+    <t>New turnover tax variable (highest value in the Index, about half of business tax revenue); CFC active 0 -&gt; 0.5</t>
   </si>
   <si>
     <t>Costa Rica</t>
@@ -173,63 +152,42 @@
     <t>Canada</t>
   </si>
   <si>
-    <t>R&amp;D credit up; digital services tax revenue enters</t>
+    <t>R&amp;D credit up</t>
   </si>
   <si>
     <t>Intangibles cost recovery 52% -&gt; 100%; machinery to 100%</t>
   </si>
   <si>
-    <t>Thin capitalisation 0.5 -&gt; 1 (EIFEL); DST flagged 2022-24</t>
-  </si>
-  <si>
     <t>Netherlands</t>
   </si>
   <si>
-    <t>R&amp;D credit up</t>
-  </si>
-  <si>
     <t>United States</t>
   </si>
   <si>
-    <t>CFC rules 0.33 -&gt; 0.67 (NCTI reaches active income); patent box 1 -&gt; 0; R&amp;D credit sharply up</t>
-  </si>
-  <si>
     <t>Austria</t>
   </si>
   <si>
-    <t>Buildings cost recovery 34% -&gt; 86%</t>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Norway</t>
+  </si>
+  <si>
+    <t>Mexico</t>
   </si>
   <si>
     <t>CFC exemptions -&gt; 0 (rate test)</t>
   </si>
   <si>
-    <t>Germany</t>
-  </si>
-  <si>
-    <t>Norway</t>
-  </si>
-  <si>
-    <t>Mexico</t>
-  </si>
-  <si>
-    <t>CFC exemptions -&gt; 0 (rate test); revenue-share denominators</t>
-  </si>
-  <si>
     <t>Finland</t>
   </si>
   <si>
-    <t>Top PIT rate 56.9% -&gt; 50.4%; machinery cost recovery 93% -&gt; 83%</t>
-  </si>
-  <si>
     <t>CFC exemptions corrected to 0</t>
   </si>
   <si>
     <t>Korea</t>
   </si>
   <si>
-    <t>Corporate rate 26.4% -&gt; 27.5%; corporate alt. minimum 4 -&gt; 5</t>
-  </si>
-  <si>
     <t>Intangibles cost recovery 74% -&gt; 81%; R&amp;D credit up</t>
   </si>
   <si>
@@ -245,10 +203,7 @@
     <t>Chile</t>
   </si>
   <si>
-    <t>Labour tax wedge up</t>
-  </si>
-  <si>
-    <t>Corporate alt. minimum 0 -&gt; 1; machinery and buildings cost recovery up</t>
+    <t>Buildings cost recovery 33.8% -&gt; 42.3% and machinery 63.3% -&gt; 70.6% (cost recovery script corrected); corporate alt. minimum 0 -&gt; 1</t>
   </si>
   <si>
     <t>Dividend WHT 35% -&gt; 17.45% (integration); CFC exemptions -&gt; 0 and active -&gt; 0</t>
@@ -257,12 +212,6 @@
     <t>Japan</t>
   </si>
   <si>
-    <t>Minimum tax 0.5 -&gt; 1 (UTPR); corporate alt. minimum 8 -&gt; 9</t>
-  </si>
-  <si>
-    <t>Corporate alt. minimum 1 -&gt; 8 (revised from source notes)</t>
-  </si>
-  <si>
     <t>Slovenia</t>
   </si>
   <si>
@@ -275,27 +224,18 @@
     <t>VAT threshold up about 20%</t>
   </si>
   <si>
-    <t>Top PIT rate 36% -&gt; 45.4%; threshold 12.3x -&gt; 1.3x average income</t>
-  </si>
-  <si>
     <t>Capital gains exemption 0 -&gt; 1 (PSH regime; full score, no asset or activity test)</t>
   </si>
   <si>
     <t>Iceland</t>
   </si>
   <si>
-    <t>VAT base broadened</t>
-  </si>
-  <si>
     <t>Revenue-share denominators (was 1.58% of GDP)</t>
   </si>
   <si>
     <t>Denmark</t>
   </si>
   <si>
-    <t>Top PIT rate 55.9% -&gt; 60.5%; threshold 1.2x -&gt; 5.4x (new top bracket)</t>
-  </si>
-  <si>
     <t>Belgium</t>
   </si>
   <si>
@@ -314,9 +254,6 @@
     <t>United Kingdom</t>
   </si>
   <si>
-    <t>Labour tax wedge down</t>
-  </si>
-  <si>
     <t>R&amp;D credit 18.75% -&gt; 18%</t>
   </si>
   <si>
@@ -326,9 +263,6 @@
     <t>Spain</t>
   </si>
   <si>
-    <t>Labour tax wedge down sharply</t>
-  </si>
-  <si>
     <t>Corporate alt. minimum 3 -&gt; 6; top PIT rate 45% -&gt; 48.6%</t>
   </si>
   <si>
@@ -341,9 +275,6 @@
     <t>Colombia</t>
   </si>
   <si>
-    <t>Minimum tax 0 -&gt; 0.5</t>
-  </si>
-  <si>
     <t>Both participation exemptions 0 -&gt; 0.5 (CHC regime)</t>
   </si>
   <si>
@@ -365,7 +296,58 @@
     <t>Applying to all countries: the two unallocable-revenue complexity measures are now expressed as shares of tax revenue rather than of GDP, and the Index now uses 43 variables rather than 42.</t>
   </si>
   <si>
-    <t>Excluded: annual drift in VAT thresholds and bases, property tax collections and revenue ratios, which move with the underlying economics rather than statute; and revisions confined to years before 2025.</t>
+    <t>Only discrete statutory changes are listed. Excluded are the labour tax wedge, VAT bases, VAT thresholds and property tax collections, which move with the underlying economics as well as with policy, and revisions confined to years before 2025.</t>
+  </si>
+  <si>
+    <t>QDMTT introduction.Corporate alt. minimum 0 -&gt; 1</t>
+  </si>
+  <si>
+    <t>QDMTT introduction. Corporate alt. minimum 0 -&gt; 1</t>
+  </si>
+  <si>
+    <t>Including Colombia's domestic minimum tax. Minimum tax 0 -&gt; 0.5</t>
+  </si>
+  <si>
+    <t>Elimination of small business rate. Corporate alt. minimum 1 -&gt; 0.</t>
+  </si>
+  <si>
+    <t>Digital services tax 1 -&gt; 0. Investment obligation, not a DST.</t>
+  </si>
+  <si>
+    <t>Corporate rate 16% -&gt; 17%; dividend WHT 16% -&gt; 17%; full expensing policy: machinery and intangibles cost recovery to 100%; R&amp;D credit up</t>
+  </si>
+  <si>
+    <t>Abolition of surcharge on capital gains. Capital gains rate 23% -&gt; 0</t>
+  </si>
+  <si>
+    <t>Corporate alt. minimum 1 -&gt; 2; digital services tax 1 -&gt; 0 (zero-rated); R&amp;D credit up</t>
+  </si>
+  <si>
+    <t>Thin capitalisation 0.5 -&gt; 1 (EIFEL)</t>
+  </si>
+  <si>
+    <t>CFC rules 0.33 -&gt; 0.67 (NCTI reaches active income); patent box 1 -&gt; 0 (FDII abolition, general export subsidy); R&amp;D credit sharply up</t>
+  </si>
+  <si>
+    <t>Buildings cost recovery 33.8% -&gt; 40.9% (correction to previous calculation); CFC exemptions -&gt; 0 (rate test)</t>
+  </si>
+  <si>
+    <t>Personal income tax cut: Top PIT rate 56.9% -&gt; 50.4%; phaseout of accelerated depreciation: machinery cost recovery 93% -&gt; 83%</t>
+  </si>
+  <si>
+    <t>Corporate rate 26.4% -&gt; 27.5%; corporate alt. minimum 4 -&gt; 5 due to QDMTT introduction</t>
+  </si>
+  <si>
+    <t>Minimum tax 0.5 -&gt; 1 (UTPR); corporate alt. minimum 8 -&gt; 9 (QDMTT)</t>
+  </si>
+  <si>
+    <t>Corporate alt. minimum 1 -&gt; 8 (revised from source notes, counting 9 unique rates based on income, revenue, and capital)</t>
+  </si>
+  <si>
+    <t>Top PIT rate 36% -&gt; 45.4%; including social contributions at the top rate threshold</t>
+  </si>
+  <si>
+    <t>New top PIT rate 55.9% -&gt; 60.5%; threshold 1.2x -&gt; 5.4x average salary (new top bracket)</t>
   </si>
 </sst>
 </file>
@@ -438,7 +420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -453,7 +435,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -787,7 +768,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{160FA06A-0FD8-4003-9416-5C914802409A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D84FA70-2011-4618-99FB-E7460CA9A0BD}">
   <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -795,9 +776,9 @@
     <col min="2" max="2" width="11.59765625" customWidth="1"/>
     <col min="3" max="3" width="10.59765625" customWidth="1"/>
     <col min="4" max="4" width="8.59765625" customWidth="1"/>
-    <col min="5" max="5" width="52.59765625" customWidth="1"/>
-    <col min="6" max="6" width="46.59765625" customWidth="1"/>
-    <col min="7" max="7" width="52.59765625" customWidth="1"/>
+    <col min="5" max="5" width="50.59765625" customWidth="1"/>
+    <col min="6" max="6" width="52.59765625" customWidth="1"/>
+    <col min="7" max="7" width="50.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
@@ -841,15 +822,15 @@
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="3">
         <f>2</f>
@@ -865,15 +846,15 @@
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="3">
         <f>3</f>
@@ -888,16 +869,16 @@
         <v>0</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>14</v>
+        <v>85</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B5" s="3">
         <f>4</f>
@@ -913,15 +894,15 @@
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4" t="s">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B6" s="3">
         <f>5</f>
@@ -936,16 +917,16 @@
         <v>0</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B7" s="3">
         <f>6</f>
@@ -962,12 +943,12 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B8" s="3">
         <f>7</f>
@@ -984,12 +965,12 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B9" s="3">
         <f>10</f>
@@ -1004,14 +985,14 @@
         <v>2</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
     </row>
     <row r="10" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B10" s="3">
         <f>8</f>
@@ -1026,16 +1007,16 @@
         <v>-1</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B11" s="3">
         <f>12</f>
@@ -1052,12 +1033,12 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B12" s="3">
         <f>11</f>
@@ -1074,12 +1055,12 @@
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B13" s="3">
         <f>9</f>
@@ -1093,19 +1074,17 @@
         <f>-3</f>
         <v>-3</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="E13" s="4"/>
       <c r="F13" s="4" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B14" s="3">
         <f>17</f>
@@ -1122,12 +1101,12 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B15" s="3">
         <f>14</f>
@@ -1142,18 +1121,18 @@
         <v>0</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B16" s="3">
         <f>13</f>
@@ -1168,18 +1147,18 @@
         <v>-2</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B17" s="3">
         <f>16</f>
@@ -1194,14 +1173,14 @@
         <v>0</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B18" s="3">
         <f>15</f>
@@ -1216,14 +1195,14 @@
         <v>-2</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>49</v>
+        <v>94</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B19" s="3">
         <f>19</f>
@@ -1239,15 +1218,13 @@
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>52</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="G19" s="4"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B20" s="3">
         <f>20</f>
@@ -1267,7 +1244,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="B21" s="3">
         <f>21</f>
@@ -1287,7 +1264,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="B22" s="3">
         <f>18</f>
@@ -1302,14 +1279,16 @@
         <v>-3</v>
       </c>
       <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
+      <c r="F22" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="G22" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B23" s="3">
         <f>24</f>
@@ -1324,16 +1303,16 @@
         <v>2</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>58</v>
+        <v>96</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="B24" s="3">
         <f>26</f>
@@ -1348,16 +1327,16 @@
         <v>3</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>61</v>
+        <v>97</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="G24" s="4"/>
     </row>
     <row r="25" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="B25" s="3">
         <f>23</f>
@@ -1373,15 +1352,15 @@
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="B26" s="3">
         <f>28</f>
@@ -1395,19 +1374,17 @@
         <f>3</f>
         <v>3</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>67</v>
-      </c>
+      <c r="E26" s="4"/>
       <c r="F26" s="4" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B27" s="3">
         <f>22</f>
@@ -1422,16 +1399,16 @@
         <v>-4</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>72</v>
+        <v>99</v>
       </c>
       <c r="G27" s="4"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="B28" s="3">
         <f>25</f>
@@ -1448,12 +1425,12 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="B29" s="3">
         <f>35</f>
@@ -1468,18 +1445,18 @@
         <v>7</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="B30" s="3">
         <f>29</f>
@@ -1493,17 +1470,15 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="E30" s="4" t="s">
-        <v>80</v>
-      </c>
+      <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="B31" s="3">
         <f>27</f>
@@ -1518,16 +1493,16 @@
         <v>-3</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="B32" s="3">
         <f>30</f>
@@ -1542,16 +1517,16 @@
         <v>-1</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="B33" s="3">
         <f>31</f>
@@ -1568,12 +1543,12 @@
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="B34" s="3">
         <f>33</f>
@@ -1588,14 +1563,14 @@
         <v>0</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="B35" s="3">
         <f>32</f>
@@ -1609,19 +1584,17 @@
         <f>-2</f>
         <v>-2</v>
       </c>
-      <c r="E35" s="4" t="s">
-        <v>90</v>
-      </c>
+      <c r="E35" s="4"/>
       <c r="F35" s="4" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="B36" s="3">
         <f>34</f>
@@ -1635,17 +1608,15 @@
         <f>-1</f>
         <v>-1</v>
       </c>
-      <c r="E36" s="4" t="s">
-        <v>94</v>
-      </c>
+      <c r="E36" s="4"/>
       <c r="F36" s="4" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="G36" s="4"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="B37" s="3">
         <f>37</f>
@@ -1659,17 +1630,15 @@
         <f>1</f>
         <v>1</v>
       </c>
-      <c r="E37" s="4" t="s">
-        <v>67</v>
-      </c>
+      <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="B38" s="3">
         <f>36</f>
@@ -1685,15 +1654,15 @@
       </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="B39" s="3">
         <f>38</f>
@@ -1708,32 +1677,32 @@
         <v>0</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="6" t="s">
-        <v>105</v>
+      <c r="A41" s="5" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="6" t="s">
-        <v>106</v>
+      <c r="A42" s="5" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A43" s="6" t="s">
-        <v>107</v>
+      <c r="A43" s="5" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{160FA06A-0FD8-4003-9416-5C914802409A}"/>
+  <autoFilter ref="A1:G1" xr:uid="{8D84FA70-2011-4618-99FB-E7460CA9A0BD}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>